<commit_message>
correction to solar and wind results
</commit_message>
<xml_diff>
--- a/Results/Phase 2/Ammonia/ammonia climate change breakdown results.xlsx
+++ b/Results/Phase 2/Ammonia/ammonia climate change breakdown results.xlsx
@@ -511,28 +511,28 @@
         <v>2.706008009890701</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1780932924736928</v>
+        <v>0.1780932924736926</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9929689668472601</v>
+        <v>0.9929689668472599</v>
       </c>
       <c r="G2" t="n">
-        <v>0.03566239416189191</v>
+        <v>0.03566239416189187</v>
       </c>
       <c r="H2" t="n">
-        <v>0.007175281641882765</v>
+        <v>0.007175281641882734</v>
       </c>
       <c r="I2" t="n">
-        <v>0.0007719950074056484</v>
+        <v>0.0007719950074052961</v>
       </c>
       <c r="J2" t="n">
-        <v>2.394597843492738e-05</v>
+        <v>2.394597843492736e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>0.05847720748751445</v>
+        <v>0.05847720748751425</v>
       </c>
       <c r="L2" t="n">
-        <v>0.0002349365622658823</v>
+        <v>0.0002349365622658821</v>
       </c>
       <c r="M2" t="n">
         <v>1.432599989730353</v>
@@ -553,28 +553,28 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2.697361362355053</v>
+        <v>2.697361362355055</v>
       </c>
       <c r="E3" t="n">
         <v>0.1768205809551257</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9903087563028564</v>
+        <v>0.9903087563028568</v>
       </c>
       <c r="G3" t="n">
-        <v>0.03494476554569712</v>
+        <v>0.03494476554569708</v>
       </c>
       <c r="H3" t="n">
-        <v>0.007080116861346226</v>
+        <v>0.007080116861346191</v>
       </c>
       <c r="I3" t="n">
-        <v>0.0007004995303756405</v>
+        <v>0.0007004995303765771</v>
       </c>
       <c r="J3" t="n">
         <v>2.350036145124532e-05</v>
       </c>
       <c r="K3" t="n">
-        <v>0.05464827279031591</v>
+        <v>0.05464827279031587</v>
       </c>
       <c r="L3" t="n">
         <v>0.0002348801108878565</v>
@@ -598,31 +598,31 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>2.692078225118515</v>
+        <v>2.692078225118516</v>
       </c>
       <c r="E4" t="n">
-        <v>0.17601201789749</v>
+        <v>0.1760120178974902</v>
       </c>
       <c r="F4" t="n">
-        <v>0.9884524837229285</v>
+        <v>0.988452483722929</v>
       </c>
       <c r="G4" t="n">
-        <v>0.03331803035568808</v>
+        <v>0.0333180303556881</v>
       </c>
       <c r="H4" t="n">
-        <v>0.006944467822133808</v>
+        <v>0.006944467822133828</v>
       </c>
       <c r="I4" t="n">
-        <v>0.0006753979506629409</v>
+        <v>0.0006753979506626061</v>
       </c>
       <c r="J4" t="n">
-        <v>2.318209564193791e-05</v>
+        <v>2.318209564193797e-05</v>
       </c>
       <c r="K4" t="n">
-        <v>0.05381789054968973</v>
+        <v>0.05381789054968984</v>
       </c>
       <c r="L4" t="n">
-        <v>0.0002347647013509868</v>
+        <v>0.0002347647013509866</v>
       </c>
       <c r="M4" t="n">
         <v>1.432599990022929</v>
@@ -649,25 +649,25 @@
         <v>0.1752534398441324</v>
       </c>
       <c r="F5" t="n">
-        <v>0.9852610815958212</v>
+        <v>0.9852610815958205</v>
       </c>
       <c r="G5" t="n">
-        <v>0.02999030026241247</v>
+        <v>0.02999030026241248</v>
       </c>
       <c r="H5" t="n">
-        <v>0.006837129168521929</v>
+        <v>0.006837129168521927</v>
       </c>
       <c r="I5" t="n">
-        <v>0.0006136757154107986</v>
+        <v>0.0006136757154116659</v>
       </c>
       <c r="J5" t="n">
-        <v>2.299585149579127e-05</v>
+        <v>2.299585149579124e-05</v>
       </c>
       <c r="K5" t="n">
-        <v>0.05372120059339941</v>
+        <v>0.05372120059339932</v>
       </c>
       <c r="L5" t="n">
-        <v>0.0002347303173188505</v>
+        <v>0.0002347303173188504</v>
       </c>
       <c r="M5" t="n">
         <v>1.432599990220732</v>
@@ -688,34 +688,34 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2.620133653935315</v>
+        <v>2.620133653935317</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1672737020697676</v>
+        <v>0.1672737020697674</v>
       </c>
       <c r="F6" t="n">
-        <v>0.9708555118184944</v>
+        <v>0.9708555118184946</v>
       </c>
       <c r="G6" t="n">
-        <v>0.009579472969610942</v>
+        <v>0.009579472969610944</v>
       </c>
       <c r="H6" t="n">
-        <v>0.006159847126158313</v>
+        <v>0.006159847126158327</v>
       </c>
       <c r="I6" t="n">
-        <v>0.0002767224467077283</v>
+        <v>0.0002767224467125274</v>
       </c>
       <c r="J6" t="n">
         <v>2.091862937066631e-05</v>
       </c>
       <c r="K6" t="n">
-        <v>0.03313277992802287</v>
+        <v>0.03313277992802285</v>
       </c>
       <c r="L6" t="n">
         <v>0.0002347073275291475</v>
       </c>
       <c r="M6" t="n">
-        <v>1.432599991619654</v>
+        <v>1.432599991619651</v>
       </c>
     </row>
     <row r="7">
@@ -736,28 +736,28 @@
         <v>2.597519110351288</v>
       </c>
       <c r="E7" t="n">
-        <v>0.1636728518731685</v>
+        <v>0.1636728518731687</v>
       </c>
       <c r="F7" t="n">
-        <v>0.9649987685818792</v>
+        <v>0.9649987685818789</v>
       </c>
       <c r="G7" t="n">
-        <v>0.002822094926071254</v>
+        <v>0.002822094926071259</v>
       </c>
       <c r="H7" t="n">
-        <v>0.005624863702515263</v>
+        <v>0.005624863702515259</v>
       </c>
       <c r="I7" t="n">
-        <v>0.0001513123084818843</v>
+        <v>0.0001513123084813068</v>
       </c>
       <c r="J7" t="n">
-        <v>1.960824023286368e-05</v>
+        <v>1.960824023286366e-05</v>
       </c>
       <c r="K7" t="n">
-        <v>0.02739523956802948</v>
+        <v>0.02739523956802942</v>
       </c>
       <c r="L7" t="n">
-        <v>0.0002343790212780716</v>
+        <v>0.0002343790212780715</v>
       </c>
       <c r="M7" t="n">
         <v>1.432599992129632</v>
@@ -781,28 +781,28 @@
         <v>2.587984265709649</v>
       </c>
       <c r="E8" t="n">
-        <v>0.1618991438890858</v>
+        <v>0.1618991438890859</v>
       </c>
       <c r="F8" t="n">
-        <v>0.9614587155740644</v>
+        <v>0.9614587155740638</v>
       </c>
       <c r="G8" t="n">
-        <v>0.001097844344738775</v>
+        <v>0.001097844344738763</v>
       </c>
       <c r="H8" t="n">
-        <v>0.005385663452816351</v>
+        <v>0.005385663452816359</v>
       </c>
       <c r="I8" t="n">
-        <v>6.80321758028241e-05</v>
+        <v>6.803217580299227e-05</v>
       </c>
       <c r="J8" t="n">
-        <v>1.876659201712198e-05</v>
+        <v>1.876659201712201e-05</v>
       </c>
       <c r="K8" t="n">
-        <v>0.02522199173979859</v>
+        <v>0.02522199173979853</v>
       </c>
       <c r="L8" t="n">
-        <v>0.000234115595307775</v>
+        <v>0.0002341155953077749</v>
       </c>
       <c r="M8" t="n">
         <v>1.432599992346017</v>
@@ -823,34 +823,34 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2.677924632695115</v>
+        <v>2.677924632695114</v>
       </c>
       <c r="E9" t="n">
-        <v>0.1742368626401197</v>
+        <v>0.1742368626401196</v>
       </c>
       <c r="F9" t="n">
-        <v>0.984981148901522</v>
+        <v>0.9849811489015222</v>
       </c>
       <c r="G9" t="n">
-        <v>0.02874552361591244</v>
+        <v>0.02874552361591243</v>
       </c>
       <c r="H9" t="n">
-        <v>0.006828133118718161</v>
+        <v>0.006828133118718166</v>
       </c>
       <c r="I9" t="n">
-        <v>0.0005570175837200272</v>
+        <v>0.0005570175837196057</v>
       </c>
       <c r="J9" t="n">
-        <v>2.289153866969132e-05</v>
+        <v>2.289153866969133e-05</v>
       </c>
       <c r="K9" t="n">
-        <v>0.04971823203443439</v>
+        <v>0.04971823203443441</v>
       </c>
       <c r="L9" t="n">
-        <v>0.0002348329240112782</v>
+        <v>0.0002348329240112783</v>
       </c>
       <c r="M9" t="n">
-        <v>1.432599990338008</v>
+        <v>1.432599990338007</v>
       </c>
     </row>
     <row r="10">
@@ -871,28 +871,28 @@
         <v>2.636845786131814</v>
       </c>
       <c r="E10" t="n">
-        <v>0.1689754325744339</v>
+        <v>0.168975432574434</v>
       </c>
       <c r="F10" t="n">
-        <v>0.9760507773250791</v>
+        <v>0.9760507773250797</v>
       </c>
       <c r="G10" t="n">
-        <v>0.01298082692668557</v>
+        <v>0.01298082692668556</v>
       </c>
       <c r="H10" t="n">
-        <v>0.006265986661075032</v>
+        <v>0.006265986661075028</v>
       </c>
       <c r="I10" t="n">
-        <v>0.000343170737963549</v>
+        <v>0.0003431707379633868</v>
       </c>
       <c r="J10" t="n">
-        <v>2.139452285257013e-05</v>
+        <v>2.139452285257009e-05</v>
       </c>
       <c r="K10" t="n">
-        <v>0.03937357249370858</v>
+        <v>0.03937357249370856</v>
       </c>
       <c r="L10" t="n">
-        <v>0.0002346336113925816</v>
+        <v>0.0002346336113925815</v>
       </c>
       <c r="M10" t="n">
         <v>1.432599991278623</v>
@@ -913,34 +913,34 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>2.597217932218061</v>
+        <v>2.597217932218059</v>
       </c>
       <c r="E11" t="n">
-        <v>0.1646952321262042</v>
+        <v>0.1646952321262041</v>
       </c>
       <c r="F11" t="n">
-        <v>0.9665055164240092</v>
+        <v>0.9665055164240086</v>
       </c>
       <c r="G11" t="n">
-        <v>0.00198182857909017</v>
+        <v>0.001981828579090161</v>
       </c>
       <c r="H11" t="n">
-        <v>0.005662860675727137</v>
+        <v>0.005662860675727147</v>
       </c>
       <c r="I11" t="n">
-        <v>0.0002120038589030011</v>
+        <v>0.0002120038589029575</v>
       </c>
       <c r="J11" t="n">
-        <v>1.967550545350044e-05</v>
+        <v>1.96755054535005e-05</v>
       </c>
       <c r="K11" t="n">
-        <v>0.02530632848182365</v>
+        <v>0.0253063284818236</v>
       </c>
       <c r="L11" t="n">
         <v>0.0002344944663335631</v>
       </c>
       <c r="M11" t="n">
-        <v>1.432599992100517</v>
+        <v>1.432599992100515</v>
       </c>
     </row>
   </sheetData>
@@ -1037,31 +1037,31 @@
         <v>1.989565906451694</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1780932924736928</v>
+        <v>0.1780932924736926</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4201944283241621</v>
+        <v>0.4201944283241618</v>
       </c>
       <c r="G2" t="n">
-        <v>0.03566239416189191</v>
+        <v>0.03566239416189187</v>
       </c>
       <c r="H2" t="n">
-        <v>0.007175281641882765</v>
+        <v>0.007175281641882734</v>
       </c>
       <c r="I2" t="n">
-        <v>0.0007719950074056484</v>
+        <v>0.0007719950074052961</v>
       </c>
       <c r="J2" t="n">
-        <v>2.394597843492738e-05</v>
+        <v>2.394597843492736e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>0.05847720748751445</v>
+        <v>0.05847720748751425</v>
       </c>
       <c r="L2" t="n">
-        <v>0.0002349365622658823</v>
+        <v>0.0002349365622658821</v>
       </c>
       <c r="M2" t="n">
-        <v>1.288932424814444</v>
+        <v>1.288932424814445</v>
       </c>
     </row>
     <row r="3">
@@ -1079,7 +1079,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1.978211186898917</v>
+        <v>1.978211186898918</v>
       </c>
       <c r="E3" t="n">
         <v>0.1768205809551257</v>
@@ -1088,19 +1088,19 @@
         <v>0.4148261456974744</v>
       </c>
       <c r="G3" t="n">
-        <v>0.03494476554569712</v>
+        <v>0.03494476554569708</v>
       </c>
       <c r="H3" t="n">
-        <v>0.007080116861346226</v>
+        <v>0.007080116861346191</v>
       </c>
       <c r="I3" t="n">
-        <v>0.0007004995303756405</v>
+        <v>0.0007004995303765771</v>
       </c>
       <c r="J3" t="n">
         <v>2.350036145124532e-05</v>
       </c>
       <c r="K3" t="n">
-        <v>0.05464827279031591</v>
+        <v>0.05464827279031587</v>
       </c>
       <c r="L3" t="n">
         <v>0.0002348801108878565</v>
@@ -1124,34 +1124,34 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1.96413308753661</v>
+        <v>1.964133087536611</v>
       </c>
       <c r="E4" t="n">
-        <v>0.17601201789749</v>
+        <v>0.1760120178974902</v>
       </c>
       <c r="F4" t="n">
-        <v>0.4041749107801645</v>
+        <v>0.404174910780165</v>
       </c>
       <c r="G4" t="n">
-        <v>0.03331803035568808</v>
+        <v>0.0333180303556881</v>
       </c>
       <c r="H4" t="n">
-        <v>0.006944467822133808</v>
+        <v>0.006944467822133828</v>
       </c>
       <c r="I4" t="n">
-        <v>0.0006753979506629409</v>
+        <v>0.0006753979506626061</v>
       </c>
       <c r="J4" t="n">
-        <v>2.318209564193791e-05</v>
+        <v>2.318209564193797e-05</v>
       </c>
       <c r="K4" t="n">
-        <v>0.05381789054968973</v>
+        <v>0.05381789054968984</v>
       </c>
       <c r="L4" t="n">
-        <v>0.0002347647013509868</v>
+        <v>0.0002347647013509866</v>
       </c>
       <c r="M4" t="n">
-        <v>1.288932425383788</v>
+        <v>1.288932425383789</v>
       </c>
     </row>
     <row r="5">
@@ -1178,25 +1178,25 @@
         <v>0.3830022013923652</v>
       </c>
       <c r="G5" t="n">
-        <v>0.02999030026241247</v>
+        <v>0.02999030026241248</v>
       </c>
       <c r="H5" t="n">
-        <v>0.006837129168521929</v>
+        <v>0.006837129168521927</v>
       </c>
       <c r="I5" t="n">
-        <v>0.0006136757154107986</v>
+        <v>0.0006136757154116659</v>
       </c>
       <c r="J5" t="n">
-        <v>2.299585149579127e-05</v>
+        <v>2.299585149579124e-05</v>
       </c>
       <c r="K5" t="n">
-        <v>0.05372120059339941</v>
+        <v>0.05372120059339932</v>
       </c>
       <c r="L5" t="n">
-        <v>0.0002347303173188505</v>
+        <v>0.0002347303173188504</v>
       </c>
       <c r="M5" t="n">
-        <v>1.288932426014233</v>
+        <v>1.288932426014232</v>
       </c>
     </row>
     <row r="6">
@@ -1214,34 +1214,34 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1.758039546909672</v>
+        <v>1.758039546909673</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1672737020697676</v>
+        <v>0.1672737020697674</v>
       </c>
       <c r="F6" t="n">
-        <v>0.2524289662042886</v>
+        <v>0.2524289662042885</v>
       </c>
       <c r="G6" t="n">
-        <v>0.009579472969610942</v>
+        <v>0.009579472969610944</v>
       </c>
       <c r="H6" t="n">
-        <v>0.006159847126158313</v>
+        <v>0.006159847126158327</v>
       </c>
       <c r="I6" t="n">
-        <v>0.0002767224467077283</v>
+        <v>0.0002767224467125274</v>
       </c>
       <c r="J6" t="n">
         <v>2.091862937066631e-05</v>
       </c>
       <c r="K6" t="n">
-        <v>0.03313277992802287</v>
+        <v>0.03313277992802285</v>
       </c>
       <c r="L6" t="n">
         <v>0.0002347073275291475</v>
       </c>
       <c r="M6" t="n">
-        <v>1.288932430208216</v>
+        <v>1.288932430208213</v>
       </c>
     </row>
     <row r="7">
@@ -1262,28 +1262,28 @@
         <v>1.697489544291927</v>
       </c>
       <c r="E7" t="n">
-        <v>0.1636728518731685</v>
+        <v>0.1636728518731687</v>
       </c>
       <c r="F7" t="n">
-        <v>0.2086367630212066</v>
+        <v>0.2086367630212067</v>
       </c>
       <c r="G7" t="n">
-        <v>0.002822094926071254</v>
+        <v>0.002822094926071259</v>
       </c>
       <c r="H7" t="n">
-        <v>0.005624863702515263</v>
+        <v>0.005624863702515259</v>
       </c>
       <c r="I7" t="n">
-        <v>0.0001513123084818843</v>
+        <v>0.0001513123084813068</v>
       </c>
       <c r="J7" t="n">
-        <v>1.960824023286368e-05</v>
+        <v>1.960824023286366e-05</v>
       </c>
       <c r="K7" t="n">
-        <v>0.02739523956802948</v>
+        <v>0.02739523956802942</v>
       </c>
       <c r="L7" t="n">
-        <v>0.0002343790212780716</v>
+        <v>0.0002343790212780715</v>
       </c>
       <c r="M7" t="n">
         <v>1.288932431630943</v>
@@ -1307,28 +1307,28 @@
         <v>1.679816484006319</v>
       </c>
       <c r="E8" t="n">
-        <v>0.1618991438890858</v>
+        <v>0.1618991438890859</v>
       </c>
       <c r="F8" t="n">
         <v>0.196958494173612</v>
       </c>
       <c r="G8" t="n">
-        <v>0.001097844344738775</v>
+        <v>0.001097844344738763</v>
       </c>
       <c r="H8" t="n">
-        <v>0.005385663452816351</v>
+        <v>0.005385663452816359</v>
       </c>
       <c r="I8" t="n">
-        <v>6.80321758028241e-05</v>
+        <v>6.803217580299227e-05</v>
       </c>
       <c r="J8" t="n">
-        <v>1.876659201712198e-05</v>
+        <v>1.876659201712201e-05</v>
       </c>
       <c r="K8" t="n">
-        <v>0.02522199173979859</v>
+        <v>0.02522199173979853</v>
       </c>
       <c r="L8" t="n">
-        <v>0.000234115595307775</v>
+        <v>0.0002341155953077749</v>
       </c>
       <c r="M8" t="n">
         <v>1.288932432043139</v>
@@ -1349,31 +1349,31 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1.923870069285613</v>
+        <v>1.923870069285612</v>
       </c>
       <c r="E9" t="n">
-        <v>0.1742368626401197</v>
+        <v>0.1742368626401196</v>
       </c>
       <c r="F9" t="n">
-        <v>0.3745941495029534</v>
+        <v>0.3745941495029533</v>
       </c>
       <c r="G9" t="n">
-        <v>0.02874552361591244</v>
+        <v>0.02874552361591243</v>
       </c>
       <c r="H9" t="n">
-        <v>0.006828133118718161</v>
+        <v>0.006828133118718166</v>
       </c>
       <c r="I9" t="n">
-        <v>0.0005570175837200272</v>
+        <v>0.0005570175837196057</v>
       </c>
       <c r="J9" t="n">
-        <v>2.289153866969132e-05</v>
+        <v>2.289153866969133e-05</v>
       </c>
       <c r="K9" t="n">
-        <v>0.04971823203443439</v>
+        <v>0.04971823203443441</v>
       </c>
       <c r="L9" t="n">
-        <v>0.0002348329240112782</v>
+        <v>0.0002348329240112783</v>
       </c>
       <c r="M9" t="n">
         <v>1.288932426327074</v>
@@ -1397,28 +1397,28 @@
         <v>1.791453194032336</v>
       </c>
       <c r="E10" t="n">
-        <v>0.1689754325744339</v>
+        <v>0.168975432574434</v>
       </c>
       <c r="F10" t="n">
         <v>0.2743257470388896</v>
       </c>
       <c r="G10" t="n">
-        <v>0.01298082692668557</v>
+        <v>0.01298082692668556</v>
       </c>
       <c r="H10" t="n">
-        <v>0.006265986661075032</v>
+        <v>0.006265986661075028</v>
       </c>
       <c r="I10" t="n">
-        <v>0.000343170737963549</v>
+        <v>0.0003431707379633868</v>
       </c>
       <c r="J10" t="n">
-        <v>2.139452285257013e-05</v>
+        <v>2.139452285257009e-05</v>
       </c>
       <c r="K10" t="n">
-        <v>0.03937357249370858</v>
+        <v>0.03937357249370856</v>
       </c>
       <c r="L10" t="n">
-        <v>0.0002346336113925816</v>
+        <v>0.0002346336113925815</v>
       </c>
       <c r="M10" t="n">
         <v>1.288932429465335</v>
@@ -1439,28 +1439,28 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1.691273365073799</v>
+        <v>1.691273365073798</v>
       </c>
       <c r="E11" t="n">
-        <v>0.1646952321262042</v>
+        <v>0.1646952321262041</v>
       </c>
       <c r="F11" t="n">
-        <v>0.2042285096361147</v>
+        <v>0.2042285096361148</v>
       </c>
       <c r="G11" t="n">
-        <v>0.00198182857909017</v>
+        <v>0.001981828579090161</v>
       </c>
       <c r="H11" t="n">
-        <v>0.005662860675727137</v>
+        <v>0.005662860675727147</v>
       </c>
       <c r="I11" t="n">
-        <v>0.0002120038589030011</v>
+        <v>0.0002120038589029575</v>
       </c>
       <c r="J11" t="n">
-        <v>1.967550545350044e-05</v>
+        <v>1.96755054535005e-05</v>
       </c>
       <c r="K11" t="n">
-        <v>0.02530632848182365</v>
+        <v>0.0253063284818236</v>
       </c>
       <c r="L11" t="n">
         <v>0.0002344944663335631</v>
@@ -1550,28 +1550,28 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.9553504935099851</v>
+        <v>0.9553504935099834</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0003273658681615044</v>
+        <v>0.0003273658681615041</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0001356635219671602</v>
+        <v>0.0001356635219671601</v>
       </c>
       <c r="G2" t="n">
-        <v>0.04834646513160136</v>
+        <v>0.04834646513160123</v>
       </c>
       <c r="H2" t="n">
-        <v>0.4027520952634854</v>
+        <v>0.4027520952634852</v>
       </c>
       <c r="I2" t="n">
-        <v>2.944450246784683e-07</v>
+        <v>2.94445024678453e-07</v>
       </c>
       <c r="J2" t="n">
-        <v>0.4953516167859343</v>
+        <v>0.4953516167859322</v>
       </c>
       <c r="K2" t="n">
-        <v>0.008436992493810691</v>
+        <v>0.008436992493811357</v>
       </c>
     </row>
     <row r="3">
@@ -1589,28 +1589,28 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.902414305993905</v>
+        <v>0.9024143059939039</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0003082283564827504</v>
+        <v>0.00030822835648275</v>
       </c>
       <c r="F3" t="n">
         <v>0.0001309144444625493</v>
       </c>
       <c r="G3" t="n">
-        <v>0.04518086496389823</v>
+        <v>0.04518086496389826</v>
       </c>
       <c r="H3" t="n">
-        <v>0.394647579692224</v>
+        <v>0.3946475796922241</v>
       </c>
       <c r="I3" t="n">
-        <v>2.887232129260151e-07</v>
+        <v>2.887232129260016e-07</v>
       </c>
       <c r="J3" t="n">
-        <v>0.4537094369522599</v>
+        <v>0.4537094369522596</v>
       </c>
       <c r="K3" t="n">
-        <v>0.008436992861364678</v>
+        <v>0.00843699286136379</v>
       </c>
     </row>
     <row r="4">
@@ -1628,25 +1628,25 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.8411212068435041</v>
+        <v>0.8411212068435057</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0003015098723325118</v>
+        <v>0.0003015098723325119</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0001266441675120467</v>
+        <v>0.0001266441675120469</v>
       </c>
       <c r="G4" t="n">
-        <v>0.04449434028587039</v>
+        <v>0.04449434028587046</v>
       </c>
       <c r="H4" t="n">
-        <v>0.3762760984270917</v>
+        <v>0.376276098427092</v>
       </c>
       <c r="I4" t="n">
-        <v>2.786224800171552e-07</v>
+        <v>2.786224800171603e-07</v>
       </c>
       <c r="J4" t="n">
-        <v>0.4114853421763624</v>
+        <v>0.4114853421763635</v>
       </c>
       <c r="K4" t="n">
         <v>0.008436993291855099</v>
@@ -1667,22 +1667,22 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.7840436879428395</v>
+        <v>0.7840436879428393</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0002922024799817145</v>
+        <v>0.0002922024799817137</v>
       </c>
       <c r="F5" t="n">
         <v>0.0001176903444903149</v>
       </c>
       <c r="G5" t="n">
-        <v>0.04441440114716642</v>
+        <v>0.04441440114716634</v>
       </c>
       <c r="H5" t="n">
-        <v>0.3386944862264652</v>
+        <v>0.3386944862264651</v>
       </c>
       <c r="I5" t="n">
-        <v>2.705928278102137e-07</v>
+        <v>2.705928278102157e-07</v>
       </c>
       <c r="J5" t="n">
         <v>0.3920876433668622</v>
@@ -1709,25 +1709,25 @@
         <v>0.4516219471413262</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0001711763025266869</v>
+        <v>0.0001711763025266872</v>
       </c>
       <c r="F6" t="n">
-        <v>5.349336338336296e-05</v>
+        <v>5.349336338336295e-05</v>
       </c>
       <c r="G6" t="n">
-        <v>0.02739277161696186</v>
+        <v>0.0273927716169619</v>
       </c>
       <c r="H6" t="n">
-        <v>0.108185468213838</v>
+        <v>0.1081854682138382</v>
       </c>
       <c r="I6" t="n">
-        <v>2.509911952282192e-07</v>
+        <v>2.509911952282323e-07</v>
       </c>
       <c r="J6" t="n">
-        <v>0.3073817897233219</v>
+        <v>0.3073817897233221</v>
       </c>
       <c r="K6" t="n">
-        <v>0.00843699693009925</v>
+        <v>0.00843699693009875</v>
       </c>
     </row>
     <row r="7">
@@ -1745,28 +1745,28 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.3049435002443067</v>
+        <v>0.3049435002443068</v>
       </c>
       <c r="E7" t="n">
         <v>0.0001392637843274556</v>
       </c>
       <c r="F7" t="n">
-        <v>3.32975745953618e-05</v>
+        <v>3.329757459536182e-05</v>
       </c>
       <c r="G7" t="n">
-        <v>0.02264921755763372</v>
+        <v>0.0226492175576337</v>
       </c>
       <c r="H7" t="n">
-        <v>0.03187123779037238</v>
+        <v>0.03187123779037239</v>
       </c>
       <c r="I7" t="n">
-        <v>1.938964378820229e-07</v>
+        <v>1.938964378820212e-07</v>
       </c>
       <c r="J7" t="n">
-        <v>0.2418132914827766</v>
+        <v>0.2418132914827777</v>
       </c>
       <c r="K7" t="n">
-        <v>0.008436998158163289</v>
+        <v>0.008436998158162345</v>
       </c>
     </row>
     <row r="8">
@@ -1784,28 +1784,28 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.2633741616726774</v>
+        <v>0.2633741616726762</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0001268136752651771</v>
+        <v>0.0001268136752651773</v>
       </c>
       <c r="F8" t="n">
         <v>2.683441427055336e-05</v>
       </c>
       <c r="G8" t="n">
-        <v>0.02085246879235921</v>
+        <v>0.02085246879235927</v>
       </c>
       <c r="H8" t="n">
-        <v>0.01239846960665351</v>
+        <v>0.01239846960665342</v>
       </c>
       <c r="I8" t="n">
-        <v>1.313381314772107e-07</v>
+        <v>1.3133813147719e-07</v>
       </c>
       <c r="J8" t="n">
-        <v>0.221532445344409</v>
+        <v>0.2215324453444089</v>
       </c>
       <c r="K8" t="n">
-        <v>0.008436998501588411</v>
+        <v>0.008436998501587412</v>
       </c>
     </row>
     <row r="9">
@@ -1823,28 +1823,28 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.7849256336739197</v>
+        <v>0.7849256336739204</v>
       </c>
       <c r="E9" t="n">
-        <v>0.0002788608290815207</v>
+        <v>0.0002788608290815211</v>
       </c>
       <c r="F9" t="n">
         <v>0.0001134446468861539</v>
       </c>
       <c r="G9" t="n">
-        <v>0.04110491719309385</v>
+        <v>0.04110491719309386</v>
       </c>
       <c r="H9" t="n">
-        <v>0.3246366414211758</v>
+        <v>0.3246366414211757</v>
       </c>
       <c r="I9" t="n">
-        <v>2.797346495780788e-07</v>
+        <v>2.797346495781052e-07</v>
       </c>
       <c r="J9" t="n">
-        <v>0.4103544959571349</v>
+        <v>0.4103544959571346</v>
       </c>
       <c r="K9" t="n">
-        <v>0.008436993891898004</v>
+        <v>0.008436993891899114</v>
       </c>
     </row>
     <row r="10">
@@ -1862,28 +1862,28 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.4964361061495565</v>
+        <v>0.4964361061495562</v>
       </c>
       <c r="E10" t="n">
-        <v>0.0002190130611853353</v>
+        <v>0.0002190130611853348</v>
       </c>
       <c r="F10" t="n">
-        <v>7.119924330083524e-05</v>
+        <v>7.119924330083512e-05</v>
       </c>
       <c r="G10" t="n">
-        <v>0.03255239317096485</v>
+        <v>0.03255239317096484</v>
       </c>
       <c r="H10" t="n">
-        <v>0.1465985491395269</v>
+        <v>0.1465985491395266</v>
       </c>
       <c r="I10" t="n">
-        <v>2.527877408564234e-07</v>
+        <v>2.527877408564025e-07</v>
       </c>
       <c r="J10" t="n">
         <v>0.3085577023136259</v>
       </c>
       <c r="K10" t="n">
-        <v>0.008436996433211774</v>
+        <v>0.008436996433211885</v>
       </c>
     </row>
     <row r="11">
@@ -1901,28 +1901,28 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.3113703044865835</v>
+        <v>0.3113703044865839</v>
       </c>
       <c r="E11" t="n">
-        <v>0.0001193015987215101</v>
+        <v>0.0001193015987215094</v>
       </c>
       <c r="F11" t="n">
-        <v>3.241086841599089e-05</v>
+        <v>3.241086841599081e-05</v>
       </c>
       <c r="G11" t="n">
-        <v>0.02092219481952109</v>
+        <v>0.02092219481952105</v>
       </c>
       <c r="H11" t="n">
-        <v>0.02238171697217529</v>
+        <v>0.02238171697217518</v>
       </c>
       <c r="I11" t="n">
-        <v>2.21351203567005e-07</v>
+        <v>2.213512035670071e-07</v>
       </c>
       <c r="J11" t="n">
-        <v>0.2594774606844535</v>
+        <v>0.2594774606844548</v>
       </c>
       <c r="K11" t="n">
-        <v>0.008436998192092537</v>
+        <v>0.008436998192091816</v>
       </c>
     </row>
   </sheetData>
@@ -2006,28 +2006,28 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1.268039716468294</v>
+        <v>1.268039716468293</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0003273658681615044</v>
+        <v>0.0003273658681615041</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0001356635219671602</v>
+        <v>0.0001356635219671601</v>
       </c>
       <c r="G2" t="n">
-        <v>0.04834646513160136</v>
+        <v>0.04834646513160123</v>
       </c>
       <c r="H2" t="n">
-        <v>0.4027520952634854</v>
+        <v>0.4027520952634852</v>
       </c>
       <c r="I2" t="n">
-        <v>2.944450246784683e-07</v>
+        <v>2.94445024678453e-07</v>
       </c>
       <c r="J2" t="n">
-        <v>0.8080408414385816</v>
+        <v>0.8080408414385806</v>
       </c>
       <c r="K2" t="n">
-        <v>0.008436990799472133</v>
+        <v>0.008436990799472799</v>
       </c>
     </row>
     <row r="3">
@@ -2048,22 +2048,22 @@
         <v>1.133248574220077</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0003082283564827504</v>
+        <v>0.00030822835648275</v>
       </c>
       <c r="F3" t="n">
         <v>0.0001309144444625493</v>
       </c>
       <c r="G3" t="n">
-        <v>0.04518086496389823</v>
+        <v>0.04518086496389826</v>
       </c>
       <c r="H3" t="n">
-        <v>0.394647579692224</v>
+        <v>0.3946475796922241</v>
       </c>
       <c r="I3" t="n">
-        <v>2.887232129260151e-07</v>
+        <v>2.887232129260016e-07</v>
       </c>
       <c r="J3" t="n">
-        <v>0.6845437064292297</v>
+        <v>0.6845437064292296</v>
       </c>
       <c r="K3" t="n">
         <v>0.008436991610566436</v>
@@ -2087,25 +2087,25 @@
         <v>1.029622127229082</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0003015098723325118</v>
+        <v>0.0003015098723325119</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0001266441675120467</v>
+        <v>0.0001266441675120469</v>
       </c>
       <c r="G4" t="n">
-        <v>0.04449434028587039</v>
+        <v>0.04449434028587046</v>
       </c>
       <c r="H4" t="n">
-        <v>0.3762760984270917</v>
+        <v>0.376276098427092</v>
       </c>
       <c r="I4" t="n">
-        <v>2.786224800171552e-07</v>
+        <v>2.786224800171603e-07</v>
       </c>
       <c r="J4" t="n">
-        <v>0.5999862635833514</v>
+        <v>0.5999862635833513</v>
       </c>
       <c r="K4" t="n">
-        <v>0.008436992270443922</v>
+        <v>0.008436992270443255</v>
       </c>
     </row>
     <row r="5">
@@ -2123,28 +2123,28 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.9439510283295476</v>
+        <v>0.9439510283295469</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0002922024799817145</v>
+        <v>0.0002922024799817137</v>
       </c>
       <c r="F5" t="n">
         <v>0.0001176903444903149</v>
       </c>
       <c r="G5" t="n">
-        <v>0.04441440114716642</v>
+        <v>0.04441440114716634</v>
       </c>
       <c r="H5" t="n">
-        <v>0.3386944862264652</v>
+        <v>0.3386944862264651</v>
       </c>
       <c r="I5" t="n">
-        <v>2.705928278102137e-07</v>
+        <v>2.705928278102157e-07</v>
       </c>
       <c r="J5" t="n">
         <v>0.551994984620045</v>
       </c>
       <c r="K5" t="n">
-        <v>0.008436992918571029</v>
+        <v>0.008436992918570585</v>
       </c>
     </row>
     <row r="6">
@@ -2162,28 +2162,28 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.5877004668660283</v>
+        <v>0.5877004668660277</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0001711763025266869</v>
+        <v>0.0001711763025266872</v>
       </c>
       <c r="F6" t="n">
-        <v>5.349336338336296e-05</v>
+        <v>5.349336338336295e-05</v>
       </c>
       <c r="G6" t="n">
-        <v>0.02739277161696186</v>
+        <v>0.0273927716169619</v>
       </c>
       <c r="H6" t="n">
-        <v>0.108185468213838</v>
+        <v>0.1081854682138382</v>
       </c>
       <c r="I6" t="n">
-        <v>2.509911952282192e-07</v>
+        <v>2.509911952282323e-07</v>
       </c>
       <c r="J6" t="n">
-        <v>0.4434603101853804</v>
+        <v>0.4434603101853801</v>
       </c>
       <c r="K6" t="n">
-        <v>0.008436996192742741</v>
+        <v>0.008436996192742297</v>
       </c>
     </row>
     <row r="7">
@@ -2201,28 +2201,28 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.4096050428682844</v>
+        <v>0.4096050428682836</v>
       </c>
       <c r="E7" t="n">
         <v>0.0001392637843274556</v>
       </c>
       <c r="F7" t="n">
-        <v>3.32975745953618e-05</v>
+        <v>3.329757459536182e-05</v>
       </c>
       <c r="G7" t="n">
-        <v>0.02264921755763372</v>
+        <v>0.0226492175576337</v>
       </c>
       <c r="H7" t="n">
-        <v>0.03187123779037238</v>
+        <v>0.03187123779037239</v>
       </c>
       <c r="I7" t="n">
-        <v>1.938964378820229e-07</v>
+        <v>1.938964378820212e-07</v>
       </c>
       <c r="J7" t="n">
-        <v>0.3464748346738724</v>
+        <v>0.3464748346738723</v>
       </c>
       <c r="K7" t="n">
-        <v>0.008436997591045214</v>
+        <v>0.008436997591044548</v>
       </c>
     </row>
     <row r="8">
@@ -2240,28 +2240,28 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.3542538837001756</v>
+        <v>0.354253883700175</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0001268136752651771</v>
+        <v>0.0001268136752651773</v>
       </c>
       <c r="F8" t="n">
         <v>2.683441427055336e-05</v>
       </c>
       <c r="G8" t="n">
-        <v>0.02085246879235921</v>
+        <v>0.02085246879235927</v>
       </c>
       <c r="H8" t="n">
-        <v>0.01239846960665351</v>
+        <v>0.01239846960665342</v>
       </c>
       <c r="I8" t="n">
-        <v>1.313381314772107e-07</v>
+        <v>1.3133813147719e-07</v>
       </c>
       <c r="J8" t="n">
-        <v>0.312412167864349</v>
+        <v>0.3124121678643487</v>
       </c>
       <c r="K8" t="n">
-        <v>0.008436998009146712</v>
+        <v>0.008436998009146379</v>
       </c>
     </row>
     <row r="9">
@@ -2279,28 +2279,28 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1.006032879990656</v>
+        <v>1.006032879990657</v>
       </c>
       <c r="E9" t="n">
-        <v>0.0002788608290815207</v>
+        <v>0.0002788608290815211</v>
       </c>
       <c r="F9" t="n">
         <v>0.0001134446468861539</v>
       </c>
       <c r="G9" t="n">
-        <v>0.04110491719309385</v>
+        <v>0.04110491719309386</v>
       </c>
       <c r="H9" t="n">
-        <v>0.3246366414211758</v>
+        <v>0.3246366414211757</v>
       </c>
       <c r="I9" t="n">
-        <v>2.797346495780788e-07</v>
+        <v>2.797346495781052e-07</v>
       </c>
       <c r="J9" t="n">
-        <v>0.6314617434719642</v>
+        <v>0.6314617434719647</v>
       </c>
       <c r="K9" t="n">
-        <v>0.008436992693805156</v>
+        <v>0.008436992693805379</v>
       </c>
     </row>
     <row r="10">
@@ -2318,28 +2318,28 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.6597957721705101</v>
+        <v>0.6597957721705089</v>
       </c>
       <c r="E10" t="n">
-        <v>0.0002190130611853353</v>
+        <v>0.0002190130611853348</v>
       </c>
       <c r="F10" t="n">
-        <v>7.119924330083524e-05</v>
+        <v>7.119924330083512e-05</v>
       </c>
       <c r="G10" t="n">
-        <v>0.03255239317096485</v>
+        <v>0.03255239317096484</v>
       </c>
       <c r="H10" t="n">
-        <v>0.1465985491395269</v>
+        <v>0.1465985491395266</v>
       </c>
       <c r="I10" t="n">
-        <v>2.527877408564234e-07</v>
+        <v>2.527877408564025e-07</v>
       </c>
       <c r="J10" t="n">
-        <v>0.4719173692197605</v>
+        <v>0.4719173692197591</v>
       </c>
       <c r="K10" t="n">
-        <v>0.00843699554803079</v>
+        <v>0.008436995548031345</v>
       </c>
     </row>
     <row r="11">
@@ -2357,28 +2357,28 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.331457899125619</v>
+        <v>0.3314578991256165</v>
       </c>
       <c r="E11" t="n">
-        <v>0.0001193015987215101</v>
+        <v>0.0001193015987215094</v>
       </c>
       <c r="F11" t="n">
-        <v>3.241086841599089e-05</v>
+        <v>3.241086841599081e-05</v>
       </c>
       <c r="G11" t="n">
-        <v>0.02092219481952109</v>
+        <v>0.02092219481952105</v>
       </c>
       <c r="H11" t="n">
-        <v>0.02238171697217529</v>
+        <v>0.02238171697217518</v>
       </c>
       <c r="I11" t="n">
-        <v>2.21351203567005e-07</v>
+        <v>2.213512035670071e-07</v>
       </c>
       <c r="J11" t="n">
-        <v>0.2795650554323349</v>
+        <v>0.2795650554323334</v>
       </c>
       <c r="K11" t="n">
-        <v>0.008436998083246661</v>
+        <v>0.008436998083245772</v>
       </c>
     </row>
   </sheetData>

</xml_diff>